<commit_message>
Restructurer le site autour du Suivi Intervenants et intégrer Sylvia.
Navigation Edito / Fichiers de travail, Prev Vid 13 vidéos, suivi des positionnements, scripts proposés lisibles, import du transcript Clarisse Sylvia et retrait de Conflits/Registre.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/site/videos_expert.xlsx
+++ b/site/videos_expert.xlsx
@@ -571,7 +571,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Bernard Yannou, Gregoire Burge</t>
+          <t>Bernard Yannou, Gregoire Burgé</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bernard Yannou, Gregoire Burge</t>
+          <t>Bernard Yannou, Gregoire Burgé</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Fatoumata Aonon, Stephanie Oger-Roussel, Yoann Montenot</t>
+          <t>Arielle Santé, Fatoumata Aonon, Stephanie Oger-Roussel, Yoann Montenot</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Fatoumata Aonon, Stephanie Oger-Roussel, Yoann Montenot</t>
+          <t>Arielle Santé, Fatoumata Aonon, Stephanie Oger-Roussel, Yoann Montenot</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Fatoumata Aonon, Stephanie Oger-Roussel, Yoann Montenot</t>
+          <t>Arielle Santé, Fatoumata Aonon, Stephanie Oger-Roussel, Yoann Montenot</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Fatoumata Aonon, Stephanie Oger-Roussel</t>
+          <t>Arielle Santé, Fatoumata Aonon, Stephanie Oger-Roussel</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Fatoumata Aonon, Stephanie Oger-Roussel</t>
+          <t>Arielle Santé, Fatoumata Aonon, Stephanie Oger-Roussel</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Pascal Corbel</t>
+          <t>Arielle Santé, Pascal Corbel</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Pascal Corbel</t>
+          <t>Arielle Santé, Pascal Corbel</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Joel Nguen, Pascal Corbel</t>
+          <t>Arielle Santé, Joël Nguen, Pascal Corbel</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Joel Nguen, Pascal Corbel</t>
+          <t>Arielle Santé, Joël Nguen, Pascal Corbel</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Bernard Yannou, Joel Nguen, Pascal Corbel</t>
+          <t>Arielle Santé, Bernard Yannou, Joël Nguen, Pascal Corbel</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Arielle Sante, Bernard Yannou, Joel Nguen, Pascal Corbel</t>
+          <t>Arielle Santé, Bernard Yannou, Joël Nguen, Pascal Corbel</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>guide_editorial_arielle-sante.doc</t>
+          <t>guide_editorial_arielle-santé.doc</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Eneli Vino, Fatoumata Aonon, Remi Wache, Soizic Lefeuvre, Virginia Branco</t>
+          <t>Eneli Vino, Fatoumata Aonon, Rémi Waché, Soizic Lefeuvre, Virginia Branco</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Eneli Vino, Fatoumata Aonon, Remi Wache, Soizic Lefeuvre, Virginia Branco</t>
+          <t>Eneli Vino, Fatoumata Aonon, Rémi Waché, Soizic Lefeuvre, Virginia Branco</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Ajouter le script reçu de Bernard pour E1.
Mettre à jour les mails de clarification et le suivi des vidéos expert après réception de la version 2 du script Bernard Yannou.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/site/videos_expert.xlsx
+++ b/site/videos_expert.xlsx
@@ -528,10 +528,14 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>EN_ATTENTE</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>RECU</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>E1.txt</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>video_expert_E1.html</t>

</xml_diff>

<commit_message>
E1 et E20 : scripts Bernard validés pour tournage.
Dernières versions déposées dans scripts_valides/, bloc Script validé sur le site et exports Word.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/site/videos_expert.xlsx
+++ b/site/videos_expert.xlsx
@@ -724,10 +724,14 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>EN_ATTENTE</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+          <t>RECU</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>E5.txt</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>video_expert_E5.html</t>
@@ -980,10 +984,14 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>EN_ATTENTE</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
+          <t>RECU</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>E10.txt</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
           <t>video_expert_E10.html</t>
@@ -1508,10 +1516,14 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>EN_ATTENTE</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>RECU</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>E20.txt</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
           <t>video_expert_E20.html</t>

</xml_diff>